<commit_message>
Fix Amplify monorepo build config
</commit_message>
<xml_diff>
--- a/setup手順.xlsx
+++ b/setup手順.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\woody\0woodyprojects\Jakalulu\04_Projects\AMOROHOUS\taskmanager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E648966F-DBFC-44CE-8C2F-C6BA582BA6BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD7CC0D8-E93F-42CC-984D-1C5F21DC4667}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="13546" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="108">
   <si>
     <t>cd C:\Users\woody\0woodyprojects\Jakalulu\04_Projects\AMOROHOUS\taskmanager</t>
   </si>
@@ -650,6 +650,21 @@
   </si>
   <si>
     <t xml:space="preserve">npm install </t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>git repository作成</t>
+    <rPh sb="14" eb="16">
+      <t>サクセイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>git commit &amp; push</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>amplifyでbuild deploy</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1114,7 +1129,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H146"/>
+  <dimension ref="A1:H152"/>
   <sheetFormatPr defaultRowHeight="17.649999999999999"/>
   <cols>
     <col min="1" max="2" width="2.5625" customWidth="1"/>
@@ -1776,14 +1791,29 @@
         <v>102</v>
       </c>
     </row>
-    <row r="145" spans="5:5">
+    <row r="145" spans="3:5">
       <c r="E145" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="146" spans="5:5">
+    <row r="146" spans="3:5">
       <c r="E146" t="s">
         <v>103</v>
+      </c>
+    </row>
+    <row r="148" spans="3:5">
+      <c r="C148" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="150" spans="3:5">
+      <c r="C150" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="152" spans="3:5">
+      <c r="C152" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>